<commit_message>
to debug oil cap
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git_repos\vervestacks_models_himanshu\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2E9DF7A-B1AA-4C1E-8855-53BF818222EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF96C6C-CFA7-445F-A9D7-9E4F99D2E224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7513" uniqueCount="1232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7514" uniqueCount="1232">
   <si>
     <t>Unit</t>
   </si>
@@ -3790,7 +3790,7 @@
     <numFmt numFmtId="165" formatCode="#.00"/>
     <numFmt numFmtId="166" formatCode="#."/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3910,8 +3910,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3927,6 +3934,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -3957,7 +3969,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
+  <cellStyleXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0">
       <protection locked="0"/>
@@ -3986,8 +3998,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -3999,8 +4012,9 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="20"/>
   </cellXfs>
-  <cellStyles count="20">
+  <cellStyles count="21">
     <cellStyle name="Date" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Fixed" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Good" xfId="3" builtinId="26"/>
@@ -4008,6 +4022,7 @@
     <cellStyle name="Heading 3" xfId="19" builtinId="18"/>
     <cellStyle name="Heading1" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Heading2" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Neutral" xfId="20" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 10" xfId="6" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
     <cellStyle name="Normal 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
@@ -4323,7 +4338,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AED5CFC-E4F3-4B66-BDF3-D607C62E9241}">
   <dimension ref="B9:H263"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="9" spans="2:8">
       <c r="B9" t="s">
@@ -9422,11 +9437,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32957E82-8232-40A9-A839-CC5F79005B92}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -9761,22 +9776,22 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10ADB714-E6AA-4E3E-B77B-62B65BA0E218}">
   <dimension ref="A1:G75"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.06640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.46484375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.53125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" thickBot="1">
+    <row r="1" spans="1:7" ht="18" thickBot="1">
       <c r="A1" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" thickTop="1" thickBot="1">
+    <row r="2" spans="1:7" ht="16.5" thickTop="1" thickBot="1">
       <c r="A2" s="6" t="s">
         <v>48</v>
       </c>
@@ -10676,16 +10691,16 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE3245E1-8745-41DD-8AE6-2F4FA19D9F1C}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.59765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -10728,9 +10743,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:H648"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -27524,14 +27539,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet31"/>
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
@@ -27636,7 +27651,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B70617-5DBA-4C59-BDF2-D5464F062DC1}">
   <dimension ref="B9:L263"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="9" spans="2:12">
       <c r="B9" t="s">
@@ -35023,27 +35038,27 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C50B696F-B355-4FC5-AD3E-AFDC509F717D}">
   <dimension ref="B1:X45"/>
-  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.59765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.19921875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.06640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.33203125" customWidth="1"/>
-    <col min="23" max="23" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.28515625" customWidth="1"/>
+    <col min="23" max="23" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:24">
@@ -36717,38 +36732,38 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet19"/>
   <dimension ref="A1:U27"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="16.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.59765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.86328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.73046875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.59765625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.1328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4.53125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.59765625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.59765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="2.1328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.73046875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="107.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="107.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="17.25" thickBot="1">
+    <row r="1" spans="1:21" ht="18" thickBot="1">
       <c r="A1" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="15" thickTop="1" thickBot="1">
+    <row r="2" spans="1:21" ht="16.5" thickTop="1" thickBot="1">
       <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
@@ -36819,6 +36834,9 @@
       </c>
       <c r="N3" t="s">
         <v>65</v>
+      </c>
+      <c r="Q3" s="9" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -37281,17 +37299,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68A8EC7F-95E3-4526-8B78-C58A96098159}">
   <dimension ref="C1:K3"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="17.53125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.19921875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.46484375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:11">
@@ -37361,17 +37379,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31D44EBE-400A-4EA2-9DA1-076783A77DFC}">
   <dimension ref="A3:S23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="19" width="19.265625" customWidth="1"/>
+    <col min="1" max="19" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:19" ht="17.25" thickBot="1">
+    <row r="3" spans="1:19" ht="18" thickBot="1">
       <c r="A3" s="5" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="15" thickTop="1" thickBot="1">
+    <row r="4" spans="1:19" ht="16.5" thickTop="1" thickBot="1">
       <c r="A4" s="6" t="s">
         <v>10</v>
       </c>
@@ -37474,12 +37492,12 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="17.25" thickBot="1">
+    <row r="10" spans="1:19" ht="18" thickBot="1">
       <c r="A10" s="5" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="15" thickTop="1" thickBot="1">
+    <row r="11" spans="1:19" ht="16.5" thickTop="1" thickBot="1">
       <c r="A11" s="6" t="s">
         <v>10</v>
       </c>
@@ -37721,10 +37739,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C47"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -38156,7 +38174,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3E766D8-7F73-4A5A-98A5-9C85D527817F}">
   <dimension ref="A1:C35"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
   </cols>
@@ -38480,11 +38498,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.59765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-12 16:52
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDAB458F-06CA-480E-B4D3-B85ED22A6DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C83BB4A-46B5-4C90-AA52-FF907BA27260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7364DDCA-9CB7-46E4-9ADC-A9B391EDCBC5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE3F82B-73DA-4BAD-A224-EF3DD0AD28D2}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{311A2D88-CDD7-4C09-8B4E-501EE8153CFE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5029804B-6E48-4270-BFC5-F719370FE23C}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-12 16:58
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C83BB4A-46B5-4C90-AA52-FF907BA27260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BABE2FBD-A23E-4084-9661-35EE1DC57AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE3F82B-73DA-4BAD-A224-EF3DD0AD28D2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C8662E5-350B-418C-AFD3-41BF36DFEBAD}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5029804B-6E48-4270-BFC5-F719370FE23C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BBC70A6-9B71-4A65-9114-17CFCB41D78C}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-12 17:07
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BABE2FBD-A23E-4084-9661-35EE1DC57AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{53607150-8E36-49F9-BCE5-0DBD82D2C91F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C8662E5-350B-418C-AFD3-41BF36DFEBAD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5F3BDF0-7070-4CC4-9170-B8A6A33DC2B5}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BBC70A6-9B71-4A65-9114-17CFCB41D78C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21DFBD24-5708-4759-8F1A-ED633BF47C25}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-12 17:16
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53607150-8E36-49F9-BCE5-0DBD82D2C91F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A7D847E-AE00-4331-855E-7B95C8C1B9D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5F3BDF0-7070-4CC4-9170-B8A6A33DC2B5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{660F9BC1-4C52-4E63-B4FF-AB1AC8050544}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21DFBD24-5708-4759-8F1A-ED633BF47C25}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25695F2C-1AE6-463E-AB15-6026A56E15A1}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-12 17:30
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A7D847E-AE00-4331-855E-7B95C8C1B9D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7100F346-7A43-44B6-9F0D-478546C72312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{660F9BC1-4C52-4E63-B4FF-AB1AC8050544}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B989F1B4-B5F4-4785-AAC6-FEC1B427736E}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25695F2C-1AE6-463E-AB15-6026A56E15A1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF2B8E21-8263-4D5B-81A0-87D5AA934554}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-12 17:48
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7100F346-7A43-44B6-9F0D-478546C72312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D47C0630-85E6-4B5E-BE17-CC4A2A1DB73D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B989F1B4-B5F4-4785-AAC6-FEC1B427736E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA673492-05D8-41B5-ADD3-6DD8FE01E9C7}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF2B8E21-8263-4D5B-81A0-87D5AA934554}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BF30621-F866-459F-8E47-DE94B452DBDD}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-12 17:57
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D47C0630-85E6-4B5E-BE17-CC4A2A1DB73D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC019558-384D-49EE-9C11-9244652F7650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA673492-05D8-41B5-ADD3-6DD8FE01E9C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15FAC4C3-2BCD-401C-B2F5-DCEBA0CEB121}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BF30621-F866-459F-8E47-DE94B452DBDD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F002604C-725E-4598-83E9-BE359EFC50DA}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-12 18:03
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC019558-384D-49EE-9C11-9244652F7650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4104218C-FCC5-4731-B724-21CC3DEF476F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15FAC4C3-2BCD-401C-B2F5-DCEBA0CEB121}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4F8D440-E358-4B25-AEA2-87E4C6C2FAB8}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F002604C-725E-4598-83E9-BE359EFC50DA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16855B27-9F40-4F51-9FC1-33023EA5A391}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-12 18:16
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4104218C-FCC5-4731-B724-21CC3DEF476F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDCCB01F-F14C-4950-A9A9-3FF5D3CA59F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4F8D440-E358-4B25-AEA2-87E4C6C2FAB8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{366636E3-69B5-4C8B-95B2-FDA3D9A833DB}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16855B27-9F40-4F51-9FC1-33023EA5A391}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8625516-DBBB-49A3-81C7-6E6C0568BD53}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>